<commit_message>
started on the cleaning and preprocessing
</commit_message>
<xml_diff>
--- a/desired_data_structure.xlsx
+++ b/desired_data_structure.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/idahelenedencker/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/idahelenedencker/Desktop/STANDBY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3EB1086-EC67-3D4F-B4C7-FEB7BFB78D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1F7A92-3E88-3848-8F13-E18CB9CF4910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9940" yWindow="500" windowWidth="18580" windowHeight="15660" xr2:uid="{35B45B0C-289D-B541-98D0-FF19E16A6D61}"/>
+    <workbookView xWindow="5720" yWindow="500" windowWidth="22780" windowHeight="15660" xr2:uid="{35B45B0C-289D-B541-98D0-FF19E16A6D61}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="52">
   <si>
     <t>authorName</t>
   </si>
@@ -183,6 +183,15 @@
   </si>
   <si>
     <t>https://www.facebook.com/photo/?fbid=643551224456012&amp;amp;set=a.215836090560863&amp;amp;__cft__[0]=AZXX3Fc6-</t>
+  </si>
+  <si>
+    <t>date_data_collection</t>
+  </si>
+  <si>
+    <t>0505</t>
+  </si>
+  <si>
+    <t>identification</t>
   </si>
 </sst>
 </file>
@@ -279,9 +288,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022 Tema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -319,7 +328,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -425,7 +434,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -567,7 +576,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -575,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB2B6628-6529-E142-B4ED-6819B6E50981}">
-  <dimension ref="A1:Z12"/>
+  <dimension ref="A1:AB12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
@@ -596,9 +605,10 @@
     <col min="23" max="23" width="16.6640625" customWidth="1"/>
     <col min="25" max="25" width="25.5" customWidth="1"/>
     <col min="26" max="26" width="15.5" customWidth="1"/>
+    <col min="27" max="27" width="23.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:28">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -677,8 +687,14 @@
       <c r="Z1" s="5" t="s">
         <v>23</v>
       </c>
+      <c r="AA1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:28">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -757,8 +773,14 @@
       <c r="Z2" s="4" t="s">
         <v>28</v>
       </c>
+      <c r="AA2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AB2">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:26">
+    <row r="3" spans="1:28">
       <c r="A3" s="4" t="s">
         <v>15</v>
       </c>
@@ -823,8 +845,11 @@
       <c r="Z3" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="AB3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:26">
+    <row r="4" spans="1:28">
       <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
@@ -889,8 +914,11 @@
       <c r="Z4" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="AB4">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="1:26">
+    <row r="5" spans="1:28">
       <c r="A5" s="4" t="s">
         <v>20</v>
       </c>
@@ -955,14 +983,17 @@
       <c r="Z5" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="AB5">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="1:26" ht="18">
+    <row r="6" spans="1:28" ht="18">
       <c r="O6" s="3"/>
     </row>
-    <row r="7" spans="1:26">
+    <row r="7" spans="1:28">
       <c r="K7" s="1"/>
     </row>
-    <row r="10" spans="1:26">
+    <row r="10" spans="1:28">
       <c r="D10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="1"/>
@@ -971,7 +1002,7 @@
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
     </row>
-    <row r="12" spans="1:26">
+    <row r="12" spans="1:28">
       <c r="H12" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
working more on preprocessing
</commit_message>
<xml_diff>
--- a/desired_data_structure.xlsx
+++ b/desired_data_structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/idahelenedencker/Desktop/STANDBY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1F7A92-3E88-3848-8F13-E18CB9CF4910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38C3B64-BF94-794C-991F-D99D3A437CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5720" yWindow="500" windowWidth="22780" windowHeight="15660" xr2:uid="{35B45B0C-289D-B541-98D0-FF19E16A6D61}"/>
+    <workbookView xWindow="2160" yWindow="500" windowWidth="22780" windowHeight="15660" xr2:uid="{35B45B0C-289D-B541-98D0-FF19E16A6D61}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="54">
   <si>
     <t>authorName</t>
   </si>
@@ -158,9 +158,6 @@
     <t>count_wow</t>
   </si>
   <si>
-    <t>type</t>
-  </si>
-  <si>
     <t>offentlig</t>
   </si>
   <si>
@@ -192,6 +189,15 @@
   </si>
   <si>
     <t>identification</t>
+  </si>
+  <si>
+    <t>offentlig_privat</t>
+  </si>
+  <si>
+    <t>name_abbreviation</t>
+  </si>
+  <si>
+    <t>BeJe</t>
   </si>
 </sst>
 </file>
@@ -584,7 +590,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB2B6628-6529-E142-B4ED-6819B6E50981}">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AC12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
@@ -606,9 +612,10 @@
     <col min="25" max="25" width="25.5" customWidth="1"/>
     <col min="26" max="26" width="15.5" customWidth="1"/>
     <col min="27" max="27" width="23.83203125" customWidth="1"/>
+    <col min="29" max="29" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28">
+    <row r="1" spans="1:29">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -619,22 +626,22 @@
         <v>3</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>33</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>2</v>
@@ -688,13 +695,16 @@
         <v>23</v>
       </c>
       <c r="AA1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="AB1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28">
+        <v>50</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -705,16 +715,16 @@
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F2" s="4">
         <v>1</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H2" s="4">
         <v>1</v>
@@ -765,7 +775,7 @@
         <v>25</v>
       </c>
       <c r="X2" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Y2" s="4" t="s">
         <v>24</v>
@@ -774,13 +784,16 @@
         <v>28</v>
       </c>
       <c r="AA2" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="AB2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:28">
+      <c r="AC2" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29">
       <c r="A3" s="4" t="s">
         <v>15</v>
       </c>
@@ -848,8 +861,11 @@
       <c r="AB3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:28">
+      <c r="AC3" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29">
       <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
@@ -917,8 +933,11 @@
       <c r="AB4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:28">
+      <c r="AC4" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29">
       <c r="A5" s="4" t="s">
         <v>20</v>
       </c>
@@ -986,14 +1005,33 @@
       <c r="AB5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:28" ht="18">
+      <c r="AC5" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" ht="18">
       <c r="O6" s="3"/>
-    </row>
-    <row r="7" spans="1:28">
+      <c r="AB6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29">
       <c r="K7" s="1"/>
-    </row>
-    <row r="10" spans="1:28">
+      <c r="AB7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29">
+      <c r="AB8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29">
+      <c r="AB9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29">
       <c r="D10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="1"/>
@@ -1001,8 +1039,16 @@
       <c r="J10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
-    </row>
-    <row r="12" spans="1:28">
+      <c r="AB10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29">
+      <c r="AB11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29">
       <c r="H12" s="2"/>
     </row>
   </sheetData>

</xml_diff>